<commit_message>
Integrate Qdrant vector search for semantic problem lookup
- Add VectorModule: embeds problems/resources via Ollama nomic-embed-text and upserts into Qdrant Cloud (dsa_sheet collection)
- Add /vector/status, /vector/reindex, /vector/search endpoints
- Auto-reindex after Excel uploads; incremental sync on problem/resource create/update/delete
- Chatbot: new search_semantic tool; search_problem tries Qdrant first with SQL ILike fallback
- Load server/.env via dotenv; extend sample sheet to 139 rows / 24 topics
- Document Qdrant setup and add qdrant service to docker-compose
</commit_message>
<xml_diff>
--- a/client/public/sample-dsa-sheet.xlsx
+++ b/client/public/sample-dsa-sheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="DSA Sheet" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D140"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,133 +457,1911 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Strings</v>
+        <v>Arrays</v>
       </c>
       <c r="B5" t="str">
-        <v>https://youtube.com/watch?v=string-theory</v>
+        <v/>
       </c>
       <c r="C5" t="str">
-        <v>https://leetcode.com/problems/longest-substring-without-repeating-characters/</v>
+        <v>https://leetcode.com/problems/contains-duplicate/</v>
       </c>
       <c r="D5" t="str">
-        <v>Medium</v>
+        <v>Easy</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Strings</v>
+        <v>Arrays</v>
       </c>
       <c r="B6" t="str">
-        <v>https://geeksforgeeks.org/string-data-structure</v>
+        <v/>
       </c>
       <c r="C6" t="str">
-        <v>https://leetcode.com/problems/valid-anagram/</v>
+        <v>https://leetcode.com/problems/maximum-subarray/</v>
       </c>
       <c r="D6" t="str">
-        <v>Easy</v>
+        <v>Medium</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Linked Lists</v>
+        <v>Arrays</v>
       </c>
       <c r="B7" t="str">
-        <v>https://youtube.com/watch?v=linked-list-theory</v>
+        <v/>
       </c>
       <c r="C7" t="str">
-        <v>https://leetcode.com/problems/reverse-linked-list/</v>
+        <v>https://leetcode.com/problems/merge-intervals/</v>
       </c>
       <c r="D7" t="str">
-        <v>Easy</v>
+        <v>Medium</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Linked Lists</v>
+        <v>Arrays</v>
       </c>
       <c r="B8" t="str">
         <v/>
       </c>
       <c r="C8" t="str">
-        <v>https://leetcode.com/problems/merge-two-sorted-lists/</v>
+        <v>https://leetcode.com/problems/jump-game/</v>
       </c>
       <c r="D8" t="str">
-        <v>Easy</v>
+        <v>Medium</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Trees</v>
+        <v>Arrays</v>
       </c>
       <c r="B9" t="str">
-        <v>https://youtube.com/watch?v=tree-theory</v>
+        <v/>
       </c>
       <c r="C9" t="str">
-        <v>https://leetcode.com/problems/maximum-depth-of-binary-tree/</v>
+        <v>https://leetcode.com/problems/next-permutation/</v>
       </c>
       <c r="D9" t="str">
-        <v>Easy</v>
+        <v>Medium</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Trees</v>
+        <v>Arrays</v>
       </c>
       <c r="B10" t="str">
-        <v>https://geeksforgeeks.org/tree-data-structure</v>
+        <v/>
       </c>
       <c r="C10" t="str">
-        <v>https://leetcode.com/problems/invert-binary-tree/</v>
+        <v>https://leetcode.com/problems/find-the-duplicate-number/</v>
       </c>
       <c r="D10" t="str">
-        <v>Easy</v>
+        <v>Medium</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Dynamic Programming</v>
+        <v>Arrays</v>
       </c>
       <c r="B11" t="str">
-        <v>https://youtube.com/watch?v=dp-theory</v>
+        <v/>
       </c>
       <c r="C11" t="str">
-        <v>https://leetcode.com/problems/climbing-stairs/</v>
+        <v>https://leetcode.com/problems/kth-largest-element-in-an-array/</v>
       </c>
       <c r="D11" t="str">
-        <v>Easy</v>
+        <v>Medium</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Dynamic Programming</v>
+        <v>Arrays</v>
       </c>
       <c r="B12" t="str">
         <v/>
       </c>
       <c r="C12" t="str">
-        <v>https://leetcode.com/problems/coin-change/</v>
+        <v>https://leetcode.com/problems/missing-number/</v>
       </c>
       <c r="D12" t="str">
-        <v>Medium</v>
+        <v>Easy</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
+        <v>Arrays</v>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v>https://leetcode.com/problems/rotate-array/</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Strings</v>
+      </c>
+      <c r="B14" t="str">
+        <v>https://youtube.com/watch?v=string-theory</v>
+      </c>
+      <c r="C14" t="str">
+        <v>https://leetcode.com/problems/longest-substring-without-repeating-characters/</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Strings</v>
+      </c>
+      <c r="B15" t="str">
+        <v>https://geeksforgeeks.org/string-data-structure</v>
+      </c>
+      <c r="C15" t="str">
+        <v>https://leetcode.com/problems/valid-anagram/</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Strings</v>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v>https://leetcode.com/problems/group-anagrams/</v>
+      </c>
+      <c r="D16" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Strings</v>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v>https://leetcode.com/problems/palindromic-substrings/</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Strings</v>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v>https://leetcode.com/problems/longest-palindromic-substring/</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Strings</v>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v>https://leetcode.com/problems/implement-strstr/</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Strings</v>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v>https://leetcode.com/problems/reverse-words-in-a-string/</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Strings</v>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v>https://leetcode.com/problems/valid-palindrome/</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Linked List</v>
+      </c>
+      <c r="B22" t="str">
+        <v>https://youtube.com/watch?v=linked-list-theory</v>
+      </c>
+      <c r="C22" t="str">
+        <v>https://leetcode.com/problems/reverse-linked-list/</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Linked List</v>
+      </c>
+      <c r="B23" t="str">
+        <v>https://geeksforgeeks.org/linked-list-data-structure</v>
+      </c>
+      <c r="C23" t="str">
+        <v>https://leetcode.com/problems/merge-two-sorted-lists/</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Linked List</v>
+      </c>
+      <c r="B24" t="str">
+        <v/>
+      </c>
+      <c r="C24" t="str">
+        <v>https://leetcode.com/problems/linked-list-cycle/</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Linked List</v>
+      </c>
+      <c r="B25" t="str">
+        <v/>
+      </c>
+      <c r="C25" t="str">
+        <v>https://leetcode.com/problems/middle-of-the-linked-list/</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Linked List</v>
+      </c>
+      <c r="B26" t="str">
+        <v/>
+      </c>
+      <c r="C26" t="str">
+        <v>https://leetcode.com/problems/remove-nth-node-from-end-of-list/</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Linked List</v>
+      </c>
+      <c r="B27" t="str">
+        <v/>
+      </c>
+      <c r="C27" t="str">
+        <v>https://leetcode.com/problems/add-two-numbers/</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Linked List</v>
+      </c>
+      <c r="B28" t="str">
+        <v/>
+      </c>
+      <c r="C28" t="str">
+        <v>https://leetcode.com/problems/copy-list-with-random-pointer/</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Linked List</v>
+      </c>
+      <c r="B29" t="str">
+        <v/>
+      </c>
+      <c r="C29" t="str">
+        <v>https://leetcode.com/problems/palindrome-linked-list/</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Linked List</v>
+      </c>
+      <c r="B30" t="str">
+        <v/>
+      </c>
+      <c r="C30" t="str">
+        <v>https://leetcode.com/problems/lru-cache/</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Linked List</v>
+      </c>
+      <c r="B31" t="str">
+        <v/>
+      </c>
+      <c r="C31" t="str">
+        <v>https://leetcode.com/problems/sort-list/</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Stack</v>
+      </c>
+      <c r="B32" t="str">
+        <v>https://youtube.com/watch?v=stack-theory</v>
+      </c>
+      <c r="C32" t="str">
+        <v>https://leetcode.com/problems/valid-parentheses/</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Stack</v>
+      </c>
+      <c r="B33" t="str">
+        <v>https://geeksforgeeks.org/stack-data-structure</v>
+      </c>
+      <c r="C33" t="str">
+        <v>https://leetcode.com/problems/min-stack/</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Stack</v>
+      </c>
+      <c r="B34" t="str">
+        <v/>
+      </c>
+      <c r="C34" t="str">
+        <v>https://leetcode.com/problems/daily-temperatures/</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Stack</v>
+      </c>
+      <c r="B35" t="str">
+        <v/>
+      </c>
+      <c r="C35" t="str">
+        <v>https://leetcode.com/problems/largest-rectangle-in-histogram/</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Stack</v>
+      </c>
+      <c r="B36" t="str">
+        <v/>
+      </c>
+      <c r="C36" t="str">
+        <v>https://leetcode.com/problems/evaluate-reverse-polish-notation/</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Stack</v>
+      </c>
+      <c r="B37" t="str">
+        <v/>
+      </c>
+      <c r="C37" t="str">
+        <v>https://leetcode.com/problems/car-fleet/</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Queue</v>
+      </c>
+      <c r="B38" t="str">
+        <v>https://youtube.com/watch?v=queue-theory</v>
+      </c>
+      <c r="C38" t="str">
+        <v>https://leetcode.com/problems/implement-stack-using-queues/</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Queue</v>
+      </c>
+      <c r="B39" t="str">
+        <v>https://geeksforgeeks.org/queue-data-structure</v>
+      </c>
+      <c r="C39" t="str">
+        <v>https://leetcode.com/problems/design-circular-queue/</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Queue</v>
+      </c>
+      <c r="B40" t="str">
+        <v/>
+      </c>
+      <c r="C40" t="str">
+        <v>https://leetcode.com/problems/number-of-recent-calls/</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Queue</v>
+      </c>
+      <c r="B41" t="str">
+        <v/>
+      </c>
+      <c r="C41" t="str">
+        <v>https://leetcode.com/problems/sliding-window-maximum/</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Queue</v>
+      </c>
+      <c r="B42" t="str">
+        <v/>
+      </c>
+      <c r="C42" t="str">
+        <v>https://leetcode.com/problems/reveal-cards-in-increasing-order/</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Binary Search</v>
+      </c>
+      <c r="B43" t="str">
+        <v>https://youtube.com/watch?v=binary-search-theory</v>
+      </c>
+      <c r="C43" t="str">
+        <v>https://leetcode.com/problems/binary-search/</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Binary Search</v>
+      </c>
+      <c r="B44" t="str">
+        <v>https://geeksforgeeks.org/binary-search</v>
+      </c>
+      <c r="C44" t="str">
+        <v>https://leetcode.com/problems/search-in-rotated-sorted-array/</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Binary Search</v>
+      </c>
+      <c r="B45" t="str">
+        <v/>
+      </c>
+      <c r="C45" t="str">
+        <v>https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Binary Search</v>
+      </c>
+      <c r="B46" t="str">
+        <v/>
+      </c>
+      <c r="C46" t="str">
+        <v>https://leetcode.com/problems/search-insert-position/</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Binary Search</v>
+      </c>
+      <c r="B47" t="str">
+        <v/>
+      </c>
+      <c r="C47" t="str">
+        <v>https://leetcode.com/problems/find-peak-element/</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Binary Search</v>
+      </c>
+      <c r="B48" t="str">
+        <v/>
+      </c>
+      <c r="C48" t="str">
+        <v>https://leetcode.com/problems/koko-eating-bananas/</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Binary Search</v>
+      </c>
+      <c r="B49" t="str">
+        <v/>
+      </c>
+      <c r="C49" t="str">
+        <v>https://leetcode.com/problems/sqrtx/</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Binary Search</v>
+      </c>
+      <c r="B50" t="str">
+        <v/>
+      </c>
+      <c r="C50" t="str">
+        <v>https://leetcode.com/problems/time-based-key-value-store/</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Recursion</v>
+      </c>
+      <c r="B51" t="str">
+        <v>https://youtube.com/watch?v=recursion-theory</v>
+      </c>
+      <c r="C51" t="str">
+        <v>https://leetcode.com/problems/powx-n/</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Recursion</v>
+      </c>
+      <c r="B52" t="str">
+        <v>https://geeksforgeeks.org/recursion</v>
+      </c>
+      <c r="C52" t="str">
+        <v>https://leetcode.com/problems/reverse-string/</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Recursion</v>
+      </c>
+      <c r="B53" t="str">
+        <v/>
+      </c>
+      <c r="C53" t="str">
+        <v>https://leetcode.com/problems/k-th-symbol-in-grammar/</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Recursion</v>
+      </c>
+      <c r="B54" t="str">
+        <v/>
+      </c>
+      <c r="C54" t="str">
+        <v>https://leetcode.com/problems/decode-string/</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Trees</v>
+      </c>
+      <c r="B55" t="str">
+        <v>https://youtube.com/watch?v=trees-theory</v>
+      </c>
+      <c r="C55" t="str">
+        <v>https://leetcode.com/problems/invert-binary-tree/</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Trees</v>
+      </c>
+      <c r="B56" t="str">
+        <v>https://geeksforgeeks.org/binary-tree-data-structure</v>
+      </c>
+      <c r="C56" t="str">
+        <v>https://leetcode.com/problems/maximum-depth-of-binary-tree/</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Trees</v>
+      </c>
+      <c r="B57" t="str">
+        <v/>
+      </c>
+      <c r="C57" t="str">
+        <v>https://leetcode.com/problems/diameter-of-binary-tree/</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Trees</v>
+      </c>
+      <c r="B58" t="str">
+        <v/>
+      </c>
+      <c r="C58" t="str">
+        <v>https://leetcode.com/problems/binary-tree-level-order-traversal/</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Trees</v>
+      </c>
+      <c r="B59" t="str">
+        <v/>
+      </c>
+      <c r="C59" t="str">
+        <v>https://leetcode.com/problems/validate-binary-search-tree/</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Trees</v>
+      </c>
+      <c r="B60" t="str">
+        <v/>
+      </c>
+      <c r="C60" t="str">
+        <v>https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-tree/</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Trees</v>
+      </c>
+      <c r="B61" t="str">
+        <v/>
+      </c>
+      <c r="C61" t="str">
+        <v>https://leetcode.com/problems/binary-tree-maximum-path-sum/</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>Trees</v>
+      </c>
+      <c r="B62" t="str">
+        <v/>
+      </c>
+      <c r="C62" t="str">
+        <v>https://leetcode.com/problems/serialize-and-deserialize-binary-tree/</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
         <v>Graphs</v>
       </c>
-      <c r="B13" t="str">
-        <v>https://youtube.com/watch?v=graph-theory</v>
-      </c>
-      <c r="C13" t="str">
+      <c r="B63" t="str">
+        <v>https://youtube.com/watch?v=graphs-theory</v>
+      </c>
+      <c r="C63" t="str">
         <v>https://leetcode.com/problems/number-of-islands/</v>
       </c>
-      <c r="D13" t="str">
+      <c r="D63" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Graphs</v>
+      </c>
+      <c r="B64" t="str">
+        <v>https://geeksforgeeks.org/graph-data-structure</v>
+      </c>
+      <c r="C64" t="str">
+        <v>https://leetcode.com/problems/clone-graph/</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>Graphs</v>
+      </c>
+      <c r="B65" t="str">
+        <v/>
+      </c>
+      <c r="C65" t="str">
+        <v>https://leetcode.com/problems/course-schedule/</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>Graphs</v>
+      </c>
+      <c r="B66" t="str">
+        <v/>
+      </c>
+      <c r="C66" t="str">
+        <v>https://leetcode.com/problems/course-schedule-ii/</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>Graphs</v>
+      </c>
+      <c r="B67" t="str">
+        <v/>
+      </c>
+      <c r="C67" t="str">
+        <v>https://leetcode.com/problems/word-ladder/</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>Graphs</v>
+      </c>
+      <c r="B68" t="str">
+        <v/>
+      </c>
+      <c r="C68" t="str">
+        <v>https://leetcode.com/problems/surrounded-regions/</v>
+      </c>
+      <c r="D68" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>Graphs</v>
+      </c>
+      <c r="B69" t="str">
+        <v/>
+      </c>
+      <c r="C69" t="str">
+        <v>https://leetcode.com/problems/network-delay-time/</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>Graphs</v>
+      </c>
+      <c r="B70" t="str">
+        <v/>
+      </c>
+      <c r="C70" t="str">
+        <v>https://leetcode.com/problems/cheapest-flights-within-k-stops/</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>Dynamic Programming</v>
+      </c>
+      <c r="B71" t="str">
+        <v>https://youtube.com/watch?v=dp-theory</v>
+      </c>
+      <c r="C71" t="str">
+        <v>https://leetcode.com/problems/climbing-stairs/</v>
+      </c>
+      <c r="D71" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>Dynamic Programming</v>
+      </c>
+      <c r="B72" t="str">
+        <v>https://geeksforgeeks.org/dynamic-programming</v>
+      </c>
+      <c r="C72" t="str">
+        <v>https://leetcode.com/problems/house-robber/</v>
+      </c>
+      <c r="D72" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>Dynamic Programming</v>
+      </c>
+      <c r="B73" t="str">
+        <v/>
+      </c>
+      <c r="C73" t="str">
+        <v>https://leetcode.com/problems/coin-change/</v>
+      </c>
+      <c r="D73" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>Dynamic Programming</v>
+      </c>
+      <c r="B74" t="str">
+        <v/>
+      </c>
+      <c r="C74" t="str">
+        <v>https://leetcode.com/problems/longest-increasing-subsequence/</v>
+      </c>
+      <c r="D74" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>Dynamic Programming</v>
+      </c>
+      <c r="B75" t="str">
+        <v/>
+      </c>
+      <c r="C75" t="str">
+        <v>https://leetcode.com/problems/partition-equal-subset-sum/</v>
+      </c>
+      <c r="D75" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>Dynamic Programming</v>
+      </c>
+      <c r="B76" t="str">
+        <v/>
+      </c>
+      <c r="C76" t="str">
+        <v>https://leetcode.com/problems/edit-distance/</v>
+      </c>
+      <c r="D76" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>Dynamic Programming</v>
+      </c>
+      <c r="B77" t="str">
+        <v/>
+      </c>
+      <c r="C77" t="str">
+        <v>https://leetcode.com/problems/unique-paths/</v>
+      </c>
+      <c r="D77" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>Dynamic Programming</v>
+      </c>
+      <c r="B78" t="str">
+        <v/>
+      </c>
+      <c r="C78" t="str">
+        <v>https://leetcode.com/problems/word-break/</v>
+      </c>
+      <c r="D78" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>Greedy Algorithms</v>
+      </c>
+      <c r="B79" t="str">
+        <v>https://youtube.com/watch?v=greedy-theory</v>
+      </c>
+      <c r="C79" t="str">
+        <v>https://leetcode.com/problems/assign-cookies/</v>
+      </c>
+      <c r="D79" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>Greedy Algorithms</v>
+      </c>
+      <c r="B80" t="str">
+        <v>https://geeksforgeeks.org/greedy-algorithms</v>
+      </c>
+      <c r="C80" t="str">
+        <v>https://leetcode.com/problems/non-overlapping-intervals/</v>
+      </c>
+      <c r="D80" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>Greedy Algorithms</v>
+      </c>
+      <c r="B81" t="str">
+        <v/>
+      </c>
+      <c r="C81" t="str">
+        <v>https://leetcode.com/problems/minimum-number-of-arrows-to-burst-balloons/</v>
+      </c>
+      <c r="D81" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>Greedy Algorithms</v>
+      </c>
+      <c r="B82" t="str">
+        <v/>
+      </c>
+      <c r="C82" t="str">
+        <v>https://leetcode.com/problems/gas-station/</v>
+      </c>
+      <c r="D82" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>Greedy Algorithms</v>
+      </c>
+      <c r="B83" t="str">
+        <v/>
+      </c>
+      <c r="C83" t="str">
+        <v>https://leetcode.com/problems/task-scheduler/</v>
+      </c>
+      <c r="D83" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>Trie</v>
+      </c>
+      <c r="B84" t="str">
+        <v>https://youtube.com/watch?v=trie-theory</v>
+      </c>
+      <c r="C84" t="str">
+        <v>https://leetcode.com/problems/implement-trie-prefix-tree/</v>
+      </c>
+      <c r="D84" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>Trie</v>
+      </c>
+      <c r="B85" t="str">
+        <v>https://geeksforgeeks.org/trie-insert-and-search</v>
+      </c>
+      <c r="C85" t="str">
+        <v>https://leetcode.com/problems/design-add-and-search-words-data-structure/</v>
+      </c>
+      <c r="D85" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>Trie</v>
+      </c>
+      <c r="B86" t="str">
+        <v/>
+      </c>
+      <c r="C86" t="str">
+        <v>https://leetcode.com/problems/word-search-ii/</v>
+      </c>
+      <c r="D86" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>Heap / Priority Queue</v>
+      </c>
+      <c r="B87" t="str">
+        <v>https://youtube.com/watch?v=heap-theory</v>
+      </c>
+      <c r="C87" t="str">
+        <v>https://leetcode.com/problems/kth-largest-element-in-a-stream/</v>
+      </c>
+      <c r="D87" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>Heap / Priority Queue</v>
+      </c>
+      <c r="B88" t="str">
+        <v>https://geeksforgeeks.org/heap-data-structure</v>
+      </c>
+      <c r="C88" t="str">
+        <v>https://leetcode.com/problems/top-k-frequent-elements/</v>
+      </c>
+      <c r="D88" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>Heap / Priority Queue</v>
+      </c>
+      <c r="B89" t="str">
+        <v/>
+      </c>
+      <c r="C89" t="str">
+        <v>https://leetcode.com/problems/merge-k-sorted-lists/</v>
+      </c>
+      <c r="D89" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>Heap / Priority Queue</v>
+      </c>
+      <c r="B90" t="str">
+        <v/>
+      </c>
+      <c r="C90" t="str">
+        <v>https://leetcode.com/problems/find-median-from-data-stream/</v>
+      </c>
+      <c r="D90" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>Heap / Priority Queue</v>
+      </c>
+      <c r="B91" t="str">
+        <v/>
+      </c>
+      <c r="C91" t="str">
+        <v>https://leetcode.com/problems/last-stone-weight/</v>
+      </c>
+      <c r="D91" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>Backtracking</v>
+      </c>
+      <c r="B92" t="str">
+        <v>https://youtube.com/watch?v=backtracking-theory</v>
+      </c>
+      <c r="C92" t="str">
+        <v>https://leetcode.com/problems/permutations/</v>
+      </c>
+      <c r="D92" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>Backtracking</v>
+      </c>
+      <c r="B93" t="str">
+        <v>https://geeksforgeeks.org/backtracking-algorithms</v>
+      </c>
+      <c r="C93" t="str">
+        <v>https://leetcode.com/problems/combination-sum/</v>
+      </c>
+      <c r="D93" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>Backtracking</v>
+      </c>
+      <c r="B94" t="str">
+        <v/>
+      </c>
+      <c r="C94" t="str">
+        <v>https://leetcode.com/problems/generate-parentheses/</v>
+      </c>
+      <c r="D94" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>Backtracking</v>
+      </c>
+      <c r="B95" t="str">
+        <v/>
+      </c>
+      <c r="C95" t="str">
+        <v>https://leetcode.com/problems/word-search/</v>
+      </c>
+      <c r="D95" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>Backtracking</v>
+      </c>
+      <c r="B96" t="str">
+        <v/>
+      </c>
+      <c r="C96" t="str">
+        <v>https://leetcode.com/problems/sudoku-solver/</v>
+      </c>
+      <c r="D96" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>Backtracking</v>
+      </c>
+      <c r="B97" t="str">
+        <v/>
+      </c>
+      <c r="C97" t="str">
+        <v>https://leetcode.com/problems/n-queens/</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>Sliding Window</v>
+      </c>
+      <c r="B98" t="str">
+        <v>https://youtube.com/watch?v=sliding-window-theory</v>
+      </c>
+      <c r="C98" t="str">
+        <v>https://leetcode.com/problems/permutation-in-string/</v>
+      </c>
+      <c r="D98" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>Sliding Window</v>
+      </c>
+      <c r="B99" t="str">
+        <v>https://geeksforgeeks.org/window-sliding-technique</v>
+      </c>
+      <c r="C99" t="str">
+        <v>https://leetcode.com/problems/minimum-window-substring/</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>Sliding Window</v>
+      </c>
+      <c r="B100" t="str">
+        <v/>
+      </c>
+      <c r="C100" t="str">
+        <v>https://leetcode.com/problems/longest-repeating-character-replacement/</v>
+      </c>
+      <c r="D100" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>Sliding Window</v>
+      </c>
+      <c r="B101" t="str">
+        <v/>
+      </c>
+      <c r="C101" t="str">
+        <v>https://leetcode.com/problems/max-consecutive-ones-iii/</v>
+      </c>
+      <c r="D101" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="str">
+        <v>Two Pointers</v>
+      </c>
+      <c r="B102" t="str">
+        <v>https://youtube.com/watch?v=two-pointers-theory</v>
+      </c>
+      <c r="C102" t="str">
+        <v>https://leetcode.com/problems/two-sum-ii-input-array-is-sorted/</v>
+      </c>
+      <c r="D102" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Two Pointers</v>
+      </c>
+      <c r="B103" t="str">
+        <v>https://geeksforgeeks.org/two-pointers-technique</v>
+      </c>
+      <c r="C103" t="str">
+        <v>https://leetcode.com/problems/3sum/</v>
+      </c>
+      <c r="D103" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="str">
+        <v>Two Pointers</v>
+      </c>
+      <c r="B104" t="str">
+        <v/>
+      </c>
+      <c r="C104" t="str">
+        <v>https://leetcode.com/problems/container-with-most-water/</v>
+      </c>
+      <c r="D104" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="str">
+        <v>Two Pointers</v>
+      </c>
+      <c r="B105" t="str">
+        <v/>
+      </c>
+      <c r="C105" t="str">
+        <v>https://leetcode.com/problems/trapping-rain-water/</v>
+      </c>
+      <c r="D105" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="str">
+        <v>Two Pointers</v>
+      </c>
+      <c r="B106" t="str">
+        <v/>
+      </c>
+      <c r="C106" t="str">
+        <v>https://leetcode.com/problems/sort-colors/</v>
+      </c>
+      <c r="D106" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="str">
+        <v>Bit Manipulation</v>
+      </c>
+      <c r="B107" t="str">
+        <v>https://youtube.com/watch?v=bit-manipulation-theory</v>
+      </c>
+      <c r="C107" t="str">
+        <v>https://leetcode.com/problems/single-number/</v>
+      </c>
+      <c r="D107" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="str">
+        <v>Bit Manipulation</v>
+      </c>
+      <c r="B108" t="str">
+        <v>https://geeksforgeeks.org/bits-manipulation-important-tactics</v>
+      </c>
+      <c r="C108" t="str">
+        <v>https://leetcode.com/problems/number-of-1-bits/</v>
+      </c>
+      <c r="D108" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="str">
+        <v>Bit Manipulation</v>
+      </c>
+      <c r="B109" t="str">
+        <v/>
+      </c>
+      <c r="C109" t="str">
+        <v>https://leetcode.com/problems/counting-bits/</v>
+      </c>
+      <c r="D109" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="str">
+        <v>Bit Manipulation</v>
+      </c>
+      <c r="B110" t="str">
+        <v/>
+      </c>
+      <c r="C110" t="str">
+        <v>https://leetcode.com/problems/reverse-bits/</v>
+      </c>
+      <c r="D110" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="str">
+        <v>Bit Manipulation</v>
+      </c>
+      <c r="B111" t="str">
+        <v/>
+      </c>
+      <c r="C111" t="str">
+        <v>https://leetcode.com/problems/sum-of-two-integers/</v>
+      </c>
+      <c r="D111" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="str">
+        <v>Math</v>
+      </c>
+      <c r="B112" t="str">
+        <v>https://youtube.com/watch?v=math-theory</v>
+      </c>
+      <c r="C112" t="str">
+        <v>https://leetcode.com/problems/reverse-integer/</v>
+      </c>
+      <c r="D112" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="str">
+        <v>Math</v>
+      </c>
+      <c r="B113" t="str">
+        <v>https://geeksforgeeks.org/mathematical-algorithms</v>
+      </c>
+      <c r="C113" t="str">
+        <v>https://leetcode.com/problems/palindrome-number/</v>
+      </c>
+      <c r="D113" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>Math</v>
+      </c>
+      <c r="B114" t="str">
+        <v/>
+      </c>
+      <c r="C114" t="str">
+        <v>https://leetcode.com/problems/happy-number/</v>
+      </c>
+      <c r="D114" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>Math</v>
+      </c>
+      <c r="B115" t="str">
+        <v/>
+      </c>
+      <c r="C115" t="str">
+        <v>https://leetcode.com/problems/count-primes/</v>
+      </c>
+      <c r="D115" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>Math</v>
+      </c>
+      <c r="B116" t="str">
+        <v/>
+      </c>
+      <c r="C116" t="str">
+        <v>https://leetcode.com/problems/roman-to-integer/</v>
+      </c>
+      <c r="D116" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>Math</v>
+      </c>
+      <c r="B117" t="str">
+        <v/>
+      </c>
+      <c r="C117" t="str">
+        <v>https://leetcode.com/problems/excel-sheet-column-number/</v>
+      </c>
+      <c r="D117" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>Segment Tree</v>
+      </c>
+      <c r="B118" t="str">
+        <v>https://youtube.com/watch?v=segment-tree-theory</v>
+      </c>
+      <c r="C118" t="str">
+        <v>https://leetcode.com/problems/range-sum-query-mutable/</v>
+      </c>
+      <c r="D118" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>Segment Tree</v>
+      </c>
+      <c r="B119" t="str">
+        <v>https://geeksforgeeks.org/segment-tree-set-1-sum-of-given-range</v>
+      </c>
+      <c r="C119" t="str">
+        <v>https://leetcode.com/problems/count-of-smaller-numbers-after-self/</v>
+      </c>
+      <c r="D119" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>Disjoint Set Union (DSU)</v>
+      </c>
+      <c r="B120" t="str">
+        <v>https://youtube.com/watch?v=dsu-theory</v>
+      </c>
+      <c r="C120" t="str">
+        <v>https://leetcode.com/problems/number-of-provinces/</v>
+      </c>
+      <c r="D120" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>Disjoint Set Union (DSU)</v>
+      </c>
+      <c r="B121" t="str">
+        <v>https://geeksforgeeks.org/disjoint-set-data-structures</v>
+      </c>
+      <c r="C121" t="str">
+        <v>https://leetcode.com/problems/redundant-connection/</v>
+      </c>
+      <c r="D121" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>Disjoint Set Union (DSU)</v>
+      </c>
+      <c r="B122" t="str">
+        <v/>
+      </c>
+      <c r="C122" t="str">
+        <v>https://leetcode.com/problems/accounts-merge/</v>
+      </c>
+      <c r="D122" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>Disjoint Set Union (DSU)</v>
+      </c>
+      <c r="B123" t="str">
+        <v/>
+      </c>
+      <c r="C123" t="str">
+        <v>https://leetcode.com/problems/longest-consecutive-sequence/</v>
+      </c>
+      <c r="D123" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>Matrix</v>
+      </c>
+      <c r="B124" t="str">
+        <v>https://youtube.com/watch?v=matrix-theory</v>
+      </c>
+      <c r="C124" t="str">
+        <v>https://leetcode.com/problems/spiral-matrix/</v>
+      </c>
+      <c r="D124" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>Matrix</v>
+      </c>
+      <c r="B125" t="str">
+        <v>https://geeksforgeeks.org/matrix-data-structure</v>
+      </c>
+      <c r="C125" t="str">
+        <v>https://leetcode.com/problems/set-matrix-zeroes/</v>
+      </c>
+      <c r="D125" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>Matrix</v>
+      </c>
+      <c r="B126" t="str">
+        <v/>
+      </c>
+      <c r="C126" t="str">
+        <v>https://leetcode.com/problems/rotate-image/</v>
+      </c>
+      <c r="D126" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>Matrix</v>
+      </c>
+      <c r="B127" t="str">
+        <v/>
+      </c>
+      <c r="C127" t="str">
+        <v>https://leetcode.com/problems/search-a-2d-matrix/</v>
+      </c>
+      <c r="D127" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>Matrix</v>
+      </c>
+      <c r="B128" t="str">
+        <v/>
+      </c>
+      <c r="C128" t="str">
+        <v>https://leetcode.com/problems/search-a-2d-matrix-ii/</v>
+      </c>
+      <c r="D128" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>Matrix</v>
+      </c>
+      <c r="B129" t="str">
+        <v/>
+      </c>
+      <c r="C129" t="str">
+        <v>https://leetcode.com/problems/transpose-matrix/</v>
+      </c>
+      <c r="D129" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>Intervals</v>
+      </c>
+      <c r="B130" t="str">
+        <v>https://youtube.com/watch?v=intervals-theory</v>
+      </c>
+      <c r="C130" t="str">
+        <v>https://leetcode.com/problems/merge-intervals/</v>
+      </c>
+      <c r="D130" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>Intervals</v>
+      </c>
+      <c r="B131" t="str">
+        <v>https://geeksforgeeks.org/merging-intervals</v>
+      </c>
+      <c r="C131" t="str">
+        <v>https://leetcode.com/problems/insert-interval/</v>
+      </c>
+      <c r="D131" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>Intervals</v>
+      </c>
+      <c r="B132" t="str">
+        <v/>
+      </c>
+      <c r="C132" t="str">
+        <v>https://leetcode.com/problems/non-overlapping-intervals/</v>
+      </c>
+      <c r="D132" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>Intervals</v>
+      </c>
+      <c r="B133" t="str">
+        <v/>
+      </c>
+      <c r="C133" t="str">
+        <v>https://leetcode.com/problems/interval-list-intersections/</v>
+      </c>
+      <c r="D133" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>Divide and Conquer</v>
+      </c>
+      <c r="B134" t="str">
+        <v>https://youtube.com/watch?v=divide-and-conquer-theory</v>
+      </c>
+      <c r="C134" t="str">
+        <v>https://leetcode.com/problems/sort-an-array/</v>
+      </c>
+      <c r="D134" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>Divide and Conquer</v>
+      </c>
+      <c r="B135" t="str">
+        <v>https://geeksforgeeks.org/divide-and-conquer</v>
+      </c>
+      <c r="C135" t="str">
+        <v>https://leetcode.com/problems/majority-element/</v>
+      </c>
+      <c r="D135" t="str">
+        <v>Easy</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>Divide and Conquer</v>
+      </c>
+      <c r="B136" t="str">
+        <v/>
+      </c>
+      <c r="C136" t="str">
+        <v>https://leetcode.com/problems/kth-largest-element-in-an-array/</v>
+      </c>
+      <c r="D136" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>Divide and Conquer</v>
+      </c>
+      <c r="B137" t="str">
+        <v/>
+      </c>
+      <c r="C137" t="str">
+        <v>https://leetcode.com/problems/powx-n/</v>
+      </c>
+      <c r="D137" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>Topological Sort</v>
+      </c>
+      <c r="B138" t="str">
+        <v>https://youtube.com/watch?v=topological-sort-theory</v>
+      </c>
+      <c r="C138" t="str">
+        <v>https://leetcode.com/problems/course-schedule-ii/</v>
+      </c>
+      <c r="D138" t="str">
+        <v>Medium</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>Topological Sort</v>
+      </c>
+      <c r="B139" t="str">
+        <v>https://geeksforgeeks.org/topological-sorting</v>
+      </c>
+      <c r="C139" t="str">
+        <v>https://leetcode.com/problems/alien-dictionary/</v>
+      </c>
+      <c r="D139" t="str">
+        <v>Hard</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>Topological Sort</v>
+      </c>
+      <c r="B140" t="str">
+        <v/>
+      </c>
+      <c r="C140" t="str">
+        <v>https://leetcode.com/problems/minimum-height-trees/</v>
+      </c>
+      <c r="D140" t="str">
         <v>Medium</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D140"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>